<commit_message>
Alteração no excel formatado
</commit_message>
<xml_diff>
--- a/data/Meta49-formatado.xlsx
+++ b/data/Meta49-formatado.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\x379975\Documents\Demandas\concluido\META-49-1\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{972D02DC-B07B-41D6-BC8B-EC8E0E9C9D44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AC8147E-3680-4AB0-A0FA-53C8244E6EDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="734" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-24285" yWindow="3630" windowWidth="21600" windowHeight="11295" tabRatio="734" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ação 3.04" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1121" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1121" uniqueCount="177">
   <si>
     <t>Fonte: ATOS</t>
   </si>
@@ -507,9 +507,6 @@
   </si>
   <si>
     <t>Freguesia do Ó/Brasilândia</t>
-  </si>
-  <si>
-    <t>FO</t>
   </si>
   <si>
     <t>Guaianases</t>
@@ -11732,7 +11729,7 @@
     </row>
     <row r="3" spans="1:16" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="113" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B3" s="113" t="s">
         <v>97</v>
@@ -12361,7 +12358,7 @@
         <v>153</v>
       </c>
       <c r="B28" s="115" t="s">
-        <v>154</v>
+        <v>109</v>
       </c>
       <c r="C28" s="114" t="s">
         <v>99</v>
@@ -12385,7 +12382,7 @@
         <v>153</v>
       </c>
       <c r="B29" s="118" t="s">
-        <v>154</v>
+        <v>109</v>
       </c>
       <c r="C29" s="117" t="s">
         <v>100</v>
@@ -12409,7 +12406,7 @@
         <v>153</v>
       </c>
       <c r="B30" s="118" t="s">
-        <v>154</v>
+        <v>109</v>
       </c>
       <c r="C30" s="117" t="s">
         <v>101</v>
@@ -12430,7 +12427,7 @@
     </row>
     <row r="31" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="114" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B31" s="115" t="s">
         <v>110</v>
@@ -12454,7 +12451,7 @@
     </row>
     <row r="32" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="117" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B32" s="118" t="s">
         <v>110</v>
@@ -12478,7 +12475,7 @@
     </row>
     <row r="33" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="117" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B33" s="118" t="s">
         <v>110</v>
@@ -12502,7 +12499,7 @@
     </row>
     <row r="34" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="114" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B34" s="115" t="s">
         <v>111</v>
@@ -12526,7 +12523,7 @@
     </row>
     <row r="35" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="117" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B35" s="118" t="s">
         <v>111</v>
@@ -12550,7 +12547,7 @@
     </row>
     <row r="36" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="117" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B36" s="118" t="s">
         <v>111</v>
@@ -12574,7 +12571,7 @@
     </row>
     <row r="37" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="114" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B37" s="115" t="s">
         <v>112</v>
@@ -12598,7 +12595,7 @@
     </row>
     <row r="38" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="117" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B38" s="118" t="s">
         <v>112</v>
@@ -12622,7 +12619,7 @@
     </row>
     <row r="39" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="117" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B39" s="118" t="s">
         <v>112</v>
@@ -12646,7 +12643,7 @@
     </row>
     <row r="40" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="114" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B40" s="115" t="s">
         <v>113</v>
@@ -12670,7 +12667,7 @@
     </row>
     <row r="41" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="117" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B41" s="118" t="s">
         <v>113</v>
@@ -12694,7 +12691,7 @@
     </row>
     <row r="42" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="117" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B42" s="118" t="s">
         <v>113</v>
@@ -12718,7 +12715,7 @@
     </row>
     <row r="43" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="114" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B43" s="115" t="s">
         <v>114</v>
@@ -12742,7 +12739,7 @@
     </row>
     <row r="44" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="117" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B44" s="118" t="s">
         <v>114</v>
@@ -12766,7 +12763,7 @@
     </row>
     <row r="45" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="117" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B45" s="118" t="s">
         <v>114</v>
@@ -12790,7 +12787,7 @@
     </row>
     <row r="46" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="114" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B46" s="115" t="s">
         <v>115</v>
@@ -12814,7 +12811,7 @@
     </row>
     <row r="47" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="117" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B47" s="118" t="s">
         <v>115</v>
@@ -12838,7 +12835,7 @@
     </row>
     <row r="48" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="117" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B48" s="118" t="s">
         <v>115</v>
@@ -12862,7 +12859,7 @@
     </row>
     <row r="49" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="114" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B49" s="115" t="s">
         <v>116</v>
@@ -12886,7 +12883,7 @@
     </row>
     <row r="50" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="117" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B50" s="118" t="s">
         <v>116</v>
@@ -12910,7 +12907,7 @@
     </row>
     <row r="51" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="117" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B51" s="118" t="s">
         <v>116</v>
@@ -12934,7 +12931,7 @@
     </row>
     <row r="52" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="114" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B52" s="115" t="s">
         <v>117</v>
@@ -12958,7 +12955,7 @@
     </row>
     <row r="53" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="117" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B53" s="118" t="s">
         <v>117</v>
@@ -12982,7 +12979,7 @@
     </row>
     <row r="54" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="117" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B54" s="118" t="s">
         <v>117</v>
@@ -13078,7 +13075,7 @@
     </row>
     <row r="58" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="114" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B58" s="115" t="s">
         <v>119</v>
@@ -13102,7 +13099,7 @@
     </row>
     <row r="59" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="117" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B59" s="118" t="s">
         <v>119</v>
@@ -13126,7 +13123,7 @@
     </row>
     <row r="60" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="117" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B60" s="118" t="s">
         <v>119</v>
@@ -13150,7 +13147,7 @@
     </row>
     <row r="61" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="114" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B61" s="115" t="s">
         <v>120</v>
@@ -13174,7 +13171,7 @@
     </row>
     <row r="62" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="117" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B62" s="118" t="s">
         <v>120</v>
@@ -13198,7 +13195,7 @@
     </row>
     <row r="63" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="117" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B63" s="118" t="s">
         <v>120</v>
@@ -13222,7 +13219,7 @@
     </row>
     <row r="64" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="114" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B64" s="115" t="s">
         <v>121</v>
@@ -13246,7 +13243,7 @@
     </row>
     <row r="65" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="117" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B65" s="118" t="s">
         <v>121</v>
@@ -13270,7 +13267,7 @@
     </row>
     <row r="66" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="117" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B66" s="118" t="s">
         <v>121</v>
@@ -13294,7 +13291,7 @@
     </row>
     <row r="67" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="114" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B67" s="115" t="s">
         <v>122</v>
@@ -13318,7 +13315,7 @@
     </row>
     <row r="68" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="117" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B68" s="118" t="s">
         <v>122</v>
@@ -13342,7 +13339,7 @@
     </row>
     <row r="69" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="117" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B69" s="118" t="s">
         <v>122</v>
@@ -13366,7 +13363,7 @@
     </row>
     <row r="70" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="114" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B70" s="115" t="s">
         <v>123</v>
@@ -13390,7 +13387,7 @@
     </row>
     <row r="71" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="117" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B71" s="118" t="s">
         <v>123</v>
@@ -13414,7 +13411,7 @@
     </row>
     <row r="72" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="117" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B72" s="118" t="s">
         <v>123</v>
@@ -13438,7 +13435,7 @@
     </row>
     <row r="73" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="114" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B73" s="115" t="s">
         <v>124</v>
@@ -13462,7 +13459,7 @@
     </row>
     <row r="74" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="117" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B74" s="118" t="s">
         <v>124</v>
@@ -13486,7 +13483,7 @@
     </row>
     <row r="75" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="117" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B75" s="118" t="s">
         <v>124</v>
@@ -13510,7 +13507,7 @@
     </row>
     <row r="76" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="114" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B76" s="115" t="s">
         <v>125</v>
@@ -13534,7 +13531,7 @@
     </row>
     <row r="77" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="117" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B77" s="118" t="s">
         <v>125</v>
@@ -13558,7 +13555,7 @@
     </row>
     <row r="78" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="117" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B78" s="118" t="s">
         <v>125</v>
@@ -13582,7 +13579,7 @@
     </row>
     <row r="79" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="114" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B79" s="115" t="s">
         <v>126</v>
@@ -13606,7 +13603,7 @@
     </row>
     <row r="80" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="117" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B80" s="118" t="s">
         <v>126</v>
@@ -13630,7 +13627,7 @@
     </row>
     <row r="81" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="117" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B81" s="118" t="s">
         <v>126</v>
@@ -13798,7 +13795,7 @@
     </row>
     <row r="88" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="114" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B88" s="115" t="s">
         <v>128</v>
@@ -13822,7 +13819,7 @@
     </row>
     <row r="89" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="117" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B89" s="118" t="s">
         <v>128</v>
@@ -13846,7 +13843,7 @@
     </row>
     <row r="90" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="117" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B90" s="118" t="s">
         <v>128</v>
@@ -13870,7 +13867,7 @@
     </row>
     <row r="91" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="114" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B91" s="115" t="s">
         <v>129</v>
@@ -13894,7 +13891,7 @@
     </row>
     <row r="92" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="117" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B92" s="118" t="s">
         <v>129</v>
@@ -13918,7 +13915,7 @@
     </row>
     <row r="93" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="117" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B93" s="118" t="s">
         <v>129</v>
@@ -13942,7 +13939,7 @@
     </row>
     <row r="94" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="114" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B94" s="115" t="s">
         <v>130</v>
@@ -13966,7 +13963,7 @@
     </row>
     <row r="95" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="117" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B95" s="118" t="s">
         <v>130</v>
@@ -13990,7 +13987,7 @@
     </row>
     <row r="96" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="117" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B96" s="118" t="s">
         <v>130</v>
@@ -14014,7 +14011,7 @@
     </row>
     <row r="97" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="114" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B97" s="115" t="s">
         <v>131</v>
@@ -14038,7 +14035,7 @@
     </row>
     <row r="98" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="117" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B98" s="118" t="s">
         <v>131</v>
@@ -14062,7 +14059,7 @@
     </row>
     <row r="99" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="117" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B99" s="118" t="s">
         <v>131</v>
@@ -14086,7 +14083,7 @@
     </row>
     <row r="100" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="123" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B100" s="124"/>
       <c r="C100" s="125"/>
@@ -14145,7 +14142,7 @@
     </row>
     <row r="101" spans="1:16" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="129" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B101" s="129"/>
       <c r="C101" s="129"/>

</xml_diff>